<commit_message>
fix(exports): use real 5P brand logo from frontend/public/logo.png for all bảng kê
DEFAULT_LOGO_PATH was pointing to a small (9KB, 293×237) placeholder image
extracted from a DAINESE sample. All bảng kê exports (Family A / B / C,
MEIKO, DAINESE) were rendering that placeholder instead of the actual 5P
brand logo users see in the web app.

- Point DEFAULT_LOGO_PATH at frontend/public/logo.png (36KB, 1280×318 px) —
  same asset the login page + header use. Fallback to the DAINESE placeholder
  only if the frontend asset is missing.
- build_company_header_block: replace hard-coded 90×90 with aspect-preserving
  sizing — constrain by 72px height, compute width from native image ratio,
  cap at 220px so wide logos don't bleed into data columns.

Verified: GLOREX customs export now embeds the real 5P logo at 220×72 px
(EMU 2095500×685800) in every sheet. File size grew from 30KB → 81KB as
expected.

Affects every export path, not just Phase 3.
</commit_message>
<xml_diff>
--- a/plans/reports/phase-03-family-c-verification/glorex-t3-2026-customs-final.xlsx
+++ b/plans/reports/phase-03-family-c-verification/glorex-t3-2026-customs-final.xlsx
@@ -233,7 +233,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="857250" cy="857250"/>
+    <ext cx="2095500" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -263,7 +263,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="857250" cy="857250"/>
+    <ext cx="2095500" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>

</xml_diff>